<commit_message>
fix: align watchlist pipeline with updated source configuration
</commit_message>
<xml_diff>
--- a/data/rules/sourceConfig.xlsx
+++ b/data/rules/sourceConfig.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Desktop/VV_Python_Project/data/rules/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5061B2B-9425-D340-9EAC-6631270D5098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AF59364-997D-48BB-B10E-883149CFF894}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8020" yWindow="8360" windowWidth="27640" windowHeight="15920" xr2:uid="{CD5289B5-C06B-194A-96AE-6288D441C4BC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{CD5289B5-C06B-194A-96AE-6288D441C4BC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
   <si>
     <t>source</t>
   </si>
@@ -71,15 +71,31 @@
   </si>
   <si>
     <t>subjectType.code</t>
+  </si>
+  <si>
+    <t>UKSL</t>
+  </si>
+  <si>
+    <t>IndividualEntityShip</t>
+  </si>
+  <si>
+    <t>UniqueID</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -113,8 +129,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -134,9 +151,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -174,7 +191,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -280,7 +297,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -422,7 +439,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -430,14 +447,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC009C7E-7FED-434A-80FD-C4CDDA6E12F9}">
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.1640625" customWidth="1"/>
     <col min="2" max="2" width="46.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -448,7 +465,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -459,7 +476,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -468,7 +485,7 @@
       </c>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -479,7 +496,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -488,6 +505,17 @@
       </c>
       <c r="C5" s="1" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>